<commit_message>
Quartz sync: Feb 18, 2025, 9:33 AM
</commit_message>
<xml_diff>
--- a/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
+++ b/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Test\Obsidian\00_Data\01_Задачи\attachments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.grigoriev\YandexDisk\Карточка MVP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2259B3-DBD4-4579-AC02-4A43C88C333F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AF6E13-0EF1-478F-9803-34B959AD6E60}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$1:$G$184</definedName>
     <definedName name="OLE_LINK1" localSheetId="0">Лист1!$E$75</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1430,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Лист1" filterMode="1">
+  <sheetPr codeName="Лист1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G184"/>
@@ -1468,7 +1468,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>0</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>8</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>9</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>10</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>11</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>12</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>13</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>14</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>15</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>16</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>17</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>18</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>19</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>20</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>21</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>22</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>23</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>24</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>25</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>26</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>27</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>29</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>30</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>31</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>37</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>38</v>
       </c>
@@ -2457,7 +2457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>43</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
         <v>44</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
         <v>45</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9">
         <v>46</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="9">
         <v>47</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="9">
         <v>48</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="9">
         <v>49</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9">
         <v>50</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="9">
         <v>51</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9">
         <v>52</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9">
         <v>53</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="9">
         <v>54</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="9">
         <v>55</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="9">
         <v>62</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="9">
         <v>66</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="9">
         <v>67</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>68</v>
       </c>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="9">
         <v>77</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="9">
         <v>79</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="9">
         <v>83</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="9">
         <v>84</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="9">
         <v>85</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="9">
         <v>86</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="9">
         <v>90</v>
       </c>
@@ -3561,7 +3561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="9">
         <v>91</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="9">
         <v>92</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="9">
         <v>102</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="9">
         <v>105</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="9">
         <v>106</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <v>108</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="9">
         <v>109</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="9">
         <v>110</v>
       </c>
@@ -4090,7 +4090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="9">
         <v>114</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="9">
         <v>120</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="9">
         <v>128</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="9">
         <v>130</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="9">
         <v>135</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="9">
         <v>137</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="9">
         <v>138</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="9">
         <v>139</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="9">
         <v>140</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="9">
         <v>141</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="9">
         <v>142</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="9">
         <v>146</v>
       </c>
@@ -4918,7 +4918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <v>150</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="9">
         <v>151</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="9">
         <v>152</v>
       </c>
@@ -4987,7 +4987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9">
         <v>153</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="9">
         <v>154</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="9">
         <v>155</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="9">
         <v>156</v>
       </c>
@@ -5079,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="9">
         <v>157</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="9">
         <v>158</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="9">
         <v>159</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="9">
         <v>160</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="9">
         <v>161</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <v>162</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="9">
         <v>163</v>
       </c>
@@ -5240,7 +5240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="9">
         <v>164</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="9">
         <v>165</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="9">
         <v>166</v>
       </c>
@@ -5309,7 +5309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="9">
         <v>167</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="9">
         <v>168</v>
       </c>
@@ -5355,7 +5355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="9">
         <v>169</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="9">
         <v>170</v>
       </c>
@@ -5401,7 +5401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="9">
         <v>171</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="9">
         <v>172</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="9">
         <v>173</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="9">
         <v>174</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="9">
         <v>175</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="9">
         <v>176</v>
       </c>
@@ -5539,7 +5539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="9">
         <v>177</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="9">
         <v>178</v>
       </c>
@@ -5585,7 +5585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="9">
         <v>179</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="9">
         <v>180</v>
       </c>
@@ -5631,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="9">
         <v>181</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="9">
         <v>182</v>
       </c>
@@ -5678,18 +5678,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="АР"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="5">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="48" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Quartz sync: Feb 18, 2025, 9:44 AM
</commit_message>
<xml_diff>
--- a/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
+++ b/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Test\Obsidian\00_Data\01_Задачи\attachments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.grigoriev\YandexDisk\Карточка MVP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2259B3-DBD4-4579-AC02-4A43C88C333F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AF6E13-0EF1-478F-9803-34B959AD6E60}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$1:$G$184</definedName>
     <definedName name="OLE_LINK1" localSheetId="0">Лист1!$E$75</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1430,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Лист1" filterMode="1">
+  <sheetPr codeName="Лист1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G184"/>
@@ -1468,7 +1468,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>0</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>8</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>9</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>10</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>11</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>12</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>13</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>14</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>15</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>16</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>17</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>18</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>19</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>20</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>21</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>22</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>23</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>24</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>25</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>26</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>27</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>29</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>30</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>31</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>37</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>38</v>
       </c>
@@ -2457,7 +2457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>43</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
         <v>44</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
         <v>45</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9">
         <v>46</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="9">
         <v>47</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="9">
         <v>48</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="9">
         <v>49</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9">
         <v>50</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="9">
         <v>51</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9">
         <v>52</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9">
         <v>53</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="9">
         <v>54</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="9">
         <v>55</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="9">
         <v>62</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="9">
         <v>66</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="9">
         <v>67</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>68</v>
       </c>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="9">
         <v>77</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="9">
         <v>79</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="9">
         <v>83</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="9">
         <v>84</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="9">
         <v>85</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="9">
         <v>86</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="9">
         <v>90</v>
       </c>
@@ -3561,7 +3561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="9">
         <v>91</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="9">
         <v>92</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="9">
         <v>102</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="9">
         <v>105</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="9">
         <v>106</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <v>108</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="9">
         <v>109</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="9">
         <v>110</v>
       </c>
@@ -4090,7 +4090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="9">
         <v>114</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="9">
         <v>120</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="9">
         <v>128</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="9">
         <v>130</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="9">
         <v>135</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="9">
         <v>137</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="9">
         <v>138</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="9">
         <v>139</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="9">
         <v>140</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="9">
         <v>141</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="9">
         <v>142</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="9">
         <v>146</v>
       </c>
@@ -4918,7 +4918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <v>150</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="9">
         <v>151</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="9">
         <v>152</v>
       </c>
@@ -4987,7 +4987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9">
         <v>153</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="9">
         <v>154</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="9">
         <v>155</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="9">
         <v>156</v>
       </c>
@@ -5079,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="9">
         <v>157</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="9">
         <v>158</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="9">
         <v>159</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="9">
         <v>160</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="9">
         <v>161</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <v>162</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="9">
         <v>163</v>
       </c>
@@ -5240,7 +5240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="9">
         <v>164</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="9">
         <v>165</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="9">
         <v>166</v>
       </c>
@@ -5309,7 +5309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="9">
         <v>167</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="9">
         <v>168</v>
       </c>
@@ -5355,7 +5355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="9">
         <v>169</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="9">
         <v>170</v>
       </c>
@@ -5401,7 +5401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="9">
         <v>171</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="9">
         <v>172</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="9">
         <v>173</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="9">
         <v>174</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="9">
         <v>175</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="9">
         <v>176</v>
       </c>
@@ -5539,7 +5539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="9">
         <v>177</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="9">
         <v>178</v>
       </c>
@@ -5585,7 +5585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="9">
         <v>179</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="9">
         <v>180</v>
       </c>
@@ -5631,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="9">
         <v>181</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="9">
         <v>182</v>
       </c>
@@ -5678,18 +5678,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="АР"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="5">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="48" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Quartz sync: Feb 18, 2025, 2:44 PM
</commit_message>
<xml_diff>
--- a/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
+++ b/content/attachments/ТУ_АТОМ-009-00-АР-КР 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.grigoriev\YandexDisk\Карточка MVP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Test\Obsidian\00_Data\01_Задачи\attachments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AF6E13-0EF1-478F-9803-34B959AD6E60}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2259B3-DBD4-4579-AC02-4A43C88C333F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$1:$G$184</definedName>
     <definedName name="OLE_LINK1" localSheetId="0">Лист1!$E$75</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1430,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Лист1">
+  <sheetPr codeName="Лист1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G184"/>
@@ -1468,7 +1468,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>0</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>8</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>9</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>10</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>11</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>12</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>13</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>14</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>15</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>16</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>17</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>18</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>19</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>20</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>21</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>22</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>23</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>24</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>25</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>26</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>27</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>29</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>30</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>31</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>37</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>38</v>
       </c>
@@ -2457,7 +2457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>43</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
         <v>44</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
         <v>45</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9">
         <v>46</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="9">
         <v>47</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="9">
         <v>48</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="9">
         <v>49</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9">
         <v>50</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="9">
         <v>51</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9">
         <v>52</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9">
         <v>53</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="9">
         <v>54</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="9">
         <v>55</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="9">
         <v>62</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="9">
         <v>66</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="9">
         <v>67</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>68</v>
       </c>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="9">
         <v>77</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="9">
         <v>79</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="9">
         <v>83</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="9">
         <v>84</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="9">
         <v>85</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="9">
         <v>86</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="9">
         <v>90</v>
       </c>
@@ -3561,7 +3561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="9">
         <v>91</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="9">
         <v>92</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="9">
         <v>102</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="9">
         <v>105</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="9">
         <v>106</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <v>108</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="9">
         <v>109</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="9">
         <v>110</v>
       </c>
@@ -4090,7 +4090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="9">
         <v>114</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="9">
         <v>120</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="9">
         <v>128</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="9">
         <v>130</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="9">
         <v>135</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="9">
         <v>137</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="9">
         <v>138</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="9">
         <v>139</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="9">
         <v>140</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="9">
         <v>141</v>
       </c>
@@ -4734,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="9">
         <v>142</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="9">
         <v>146</v>
       </c>
@@ -4918,7 +4918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <v>150</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="9">
         <v>151</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="9">
         <v>152</v>
       </c>
@@ -4987,7 +4987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9">
         <v>153</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="9">
         <v>154</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="9">
         <v>155</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="9">
         <v>156</v>
       </c>
@@ -5079,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="9">
         <v>157</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="9">
         <v>158</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="9">
         <v>159</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="9">
         <v>160</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="9">
         <v>161</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <v>162</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="9">
         <v>163</v>
       </c>
@@ -5240,7 +5240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="9">
         <v>164</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="9">
         <v>165</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="9">
         <v>166</v>
       </c>
@@ -5309,7 +5309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="9">
         <v>167</v>
       </c>
@@ -5332,7 +5332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="9">
         <v>168</v>
       </c>
@@ -5355,7 +5355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="9">
         <v>169</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="9">
         <v>170</v>
       </c>
@@ -5401,7 +5401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="9">
         <v>171</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="9">
         <v>172</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="9">
         <v>173</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="9">
         <v>174</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="9">
         <v>175</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="9">
         <v>176</v>
       </c>
@@ -5539,7 +5539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="9">
         <v>177</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="9">
         <v>178</v>
       </c>
@@ -5585,7 +5585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="9">
         <v>179</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="9">
         <v>180</v>
       </c>
@@ -5631,7 +5631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="9">
         <v>181</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="9">
         <v>182</v>
       </c>
@@ -5678,7 +5678,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G184" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="АР"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="48" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>